<commit_message>
feat: 规则工作簿版式固化成规范 (style.py) + rule-sheet format 子命令
- 新模块 style.py 一处定义版式: 列类型配色 (输入蓝 / 输出绿 / 说明黄 / ID 灰表头)、按内容定宽
  (中文算 2, 每类列有上下限)、超宽换行并显式写行高、冻结到 ID 列之右、= 开头的格存文本、日期 yyyy-mm-dd;
  表头定位复用 loaders._parse_header, 与加载器永远一个答案
- rule-sheet format 规则.xlsx [-o 路径]: 先 load_rules 校验结构再套版式, 默认原地改写, 被占用直接报错不写副本
- 三个样例生成脚本删掉各自复制的样式代码和手调列宽, 只写内容; 去掉 PEP 723 头 (要 import rule_sheet.style),
  改用 uv run python 运行; 样例 xlsx 重新生成, 内容不变 (全部测试仍绿)
- 输出文件的列宽改用同一个 display_width (中文算 2), 原来 len*1.6 对中英混排不准
- tests/test_style.py: 样例对照规范常量校验、format 幂等 / 不改语义 / 结构错报加载器原话、CLI
- 文档: 使用指南 3.6 版式规范表与 format 命令、README、设计架构 5.14 与模块表、CLAUDE.md

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018S3X45xKo7kmWf6HK71f2W
</commit_message>
<xml_diff>
--- a/examples/customer-sync/客户主表.xlsx
+++ b/examples/customer-sync/客户主表.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,7 @@
     <font>
       <b val="1"/>
     </font>
+    <font/>
   </fonts>
   <fills count="3">
     <fill>
@@ -73,16 +74,16 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -453,11 +454,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>

</xml_diff>